<commit_message>
added results to gitignore
</commit_message>
<xml_diff>
--- a/results/Metrics.xlsx
+++ b/results/Metrics.xlsx
@@ -2,19 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
-  <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bavra\Desktop\image-unbluring\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7141DBD-A8C2-48FE-AAB1-534C89726EA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{254BCF37-35D0-4843-8EE2-72A9515DDEB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{9E8781EB-8CA8-4CA7-9ABE-25F10890F6BB}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{9E8781EB-8CA8-4CA7-9ABE-25F10890F6BB}"/>
   </bookViews>
   <sheets>
-    <sheet name="Gauss-Seidel" sheetId="2" r:id="rId1"/>
-    <sheet name="Jacobi" sheetId="1" r:id="rId2"/>
+    <sheet name="Jacobi" sheetId="5" r:id="rId1"/>
+    <sheet name="Gauss-Seidel" sheetId="4" r:id="rId2"/>
+    <sheet name="SOR" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,12 +36,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="3">
   <si>
     <t>Number of Iterations</t>
   </si>
   <si>
     <t>MSE</t>
+  </si>
+  <si>
+    <t>Omega</t>
   </si>
 </sst>
 </file>
@@ -64,15 +68,13 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -91,8 +93,14 @@
         <bgColor theme="4" tint="0.79998168889431442"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -101,8 +109,23 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
-      <right/>
+      <right style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </right>
       <top style="thin">
         <color theme="4" tint="0.39997558519241921"/>
       </top>
@@ -115,96 +138,51 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="4">
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79998168889431442"/>
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </left>
-      </border>
+      <alignment horizontal="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -239,27 +217,13 @@
           <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
           <a:lstStyle/>
           <a:p>
-            <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="ctr" defTabSz="914400" rtl="0" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
-              <a:lnSpc>
-                <a:spcPct val="100000"/>
-              </a:lnSpc>
-              <a:spcBef>
-                <a:spcPts val="0"/>
-              </a:spcBef>
-              <a:spcAft>
-                <a:spcPts val="0"/>
-              </a:spcAft>
-              <a:buClrTx/>
-              <a:buSzTx/>
-              <a:buFontTx/>
-              <a:buNone/>
-              <a:tabLst/>
+            <a:pPr>
               <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
-                  <a:sysClr val="windowText" lastClr="000000">
+                  <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
                     <a:lumOff val="35000"/>
-                  </a:sysClr>
+                  </a:schemeClr>
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
                 <a:ea typeface="+mn-ea"/>
@@ -267,20 +231,14 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-                <a:solidFill>
-                  <a:sysClr val="windowText" lastClr="000000">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:sysClr>
-                </a:solidFill>
-              </a:rPr>
-              <a:t>MSE by Number Of Iterations (Gauss-Seidel)</a:t>
+              <a:rPr lang="en-GB"/>
+              <a:t>MSE by</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="en-GB"/>
-              <a:t> </a:t>
+              <a:rPr lang="en-GB" baseline="0"/>
+              <a:t> Number of Iterations (Jacobi Method)</a:t>
             </a:r>
+            <a:endParaRPr lang="en-GB"/>
           </a:p>
         </c:rich>
       </c:tx>
@@ -296,27 +254,13 @@
         <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
         <a:lstStyle/>
         <a:p>
-          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="ctr" defTabSz="914400" rtl="0" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-            <a:spcBef>
-              <a:spcPts val="0"/>
-            </a:spcBef>
-            <a:spcAft>
-              <a:spcPts val="0"/>
-            </a:spcAft>
-            <a:buClrTx/>
-            <a:buSzTx/>
-            <a:buFontTx/>
-            <a:buNone/>
-            <a:tabLst/>
+          <a:pPr>
             <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000">
+                <a:schemeClr val="tx1">
                   <a:lumMod val="65000"/>
                   <a:lumOff val="35000"/>
-                </a:sysClr>
+                </a:schemeClr>
               </a:solidFill>
               <a:latin typeface="+mn-lt"/>
               <a:ea typeface="+mn-ea"/>
@@ -339,7 +283,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Gauss-Seidel'!$B$1</c:f>
+              <c:f>Jacobi!$B$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -350,7 +294,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent1"/>
+              <a:srgbClr val="FF0000"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -388,7 +332,6 @@
                 <a:endParaRPr lang="en-US"/>
               </a:p>
             </c:txPr>
-            <c:dLblPos val="outEnd"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="1"/>
             <c:showCatName val="0"/>
@@ -418,7 +361,7 @@
           </c:dLbls>
           <c:cat>
             <c:numRef>
-              <c:f>'Gauss-Seidel'!$A$2:$A$6</c:f>
+              <c:f>Jacobi!$A$2:$A$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -442,38 +385,37 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Gauss-Seidel'!$B$2:$B$6</c:f>
+              <c:f>Jacobi!$B$2:$B$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>45.213999999999999</c:v>
+                  <c:v>42.866999999999997</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>58.094999999999999</c:v>
+                  <c:v>48.762999999999998</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>64.718000000000004</c:v>
+                  <c:v>54.674999999999997</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>68.376000000000005</c:v>
+                  <c:v>59.201000000000001</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>70.561000000000007</c:v>
+                  <c:v>62.613</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-A242-4499-BC67-D30FC3C8FD81}"/>
+              <c16:uniqueId val="{00000000-FC81-4861-9A96-97B8CA84C857}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:dLbls>
-          <c:dLblPos val="outEnd"/>
           <c:showLegendKey val="0"/>
-          <c:showVal val="1"/>
+          <c:showVal val="0"/>
           <c:showCatName val="0"/>
           <c:showSerName val="0"/>
           <c:showPercent val="0"/>
@@ -481,71 +423,16 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="165858447"/>
-        <c:axId val="165854127"/>
+        <c:axId val="365176239"/>
+        <c:axId val="365191119"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="165858447"/>
+        <c:axId val="365176239"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="65000"/>
-                        <a:lumOff val="35000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr lang="en-GB"/>
-                  <a:t>Number of Iterations</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
-        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -583,7 +470,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="165854127"/>
+        <c:crossAx val="365191119"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -591,7 +478,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="165854127"/>
+        <c:axId val="365191119"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -611,66 +498,6 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="65000"/>
-                        <a:lumOff val="35000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr lang="en-GB"/>
-                  <a:t>Mean</a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="en-GB" baseline="0"/>
-                  <a:t> Squared Error (MSE)</a:t>
-                </a:r>
-                <a:endParaRPr lang="en-GB"/>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
-        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -702,7 +529,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="165858447"/>
+        <c:crossAx val="365176239"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -785,14 +612,13 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US"/>
-              <a:t>MSE b</a:t>
+              <a:rPr lang="en-GB"/>
+              <a:t>MSE by Number of Iterations (Gauss-Seidel</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="en-US" baseline="0"/>
-              <a:t>y Number Of Iterations (Jacobi)</a:t>
+              <a:rPr lang="en-GB" baseline="0"/>
+              <a:t> Method)</a:t>
             </a:r>
-            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:rich>
       </c:tx>
@@ -837,7 +663,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Jacobi!$B$1</c:f>
+              <c:f>'Gauss-Seidel'!$B$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -856,67 +682,9 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
-          <c:dLbls>
-            <c:spPr>
-              <a:noFill/>
-              <a:ln>
-                <a:noFill/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-                <a:spAutoFit/>
-              </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="75000"/>
-                        <a:lumOff val="25000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:endParaRPr lang="en-US"/>
-              </a:p>
-            </c:txPr>
-            <c:dLblPos val="outEnd"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showBubbleSize val="0"/>
-            <c:showLeaderLines val="0"/>
-            <c:extLst>
-              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="1"/>
-                <c15:leaderLines>
-                  <c:spPr>
-                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="35000"/>
-                          <a:lumOff val="65000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:round/>
-                    </a:ln>
-                    <a:effectLst/>
-                  </c:spPr>
-                </c15:leaderLines>
-              </c:ext>
-            </c:extLst>
-          </c:dLbls>
           <c:cat>
             <c:numRef>
-              <c:f>Jacobi!$A$2:$A$6</c:f>
+              <c:f>'Gauss-Seidel'!$A$2:$A$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -940,38 +708,37 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Jacobi!$B$2:$B$6</c:f>
+              <c:f>'Gauss-Seidel'!$B$2:$B$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>42.866999999999997</c:v>
+                  <c:v>45.213999999999999</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>48.762999999999998</c:v>
+                  <c:v>58.094999999999999</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>54.674999999999997</c:v>
+                  <c:v>64.718000000000004</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>59.201000000000001</c:v>
+                  <c:v>68.376000000000005</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>62.613</c:v>
+                  <c:v>70.561000000000007</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-3F47-4F85-B2BC-352F1D23A157}"/>
+              <c16:uniqueId val="{00000000-BFA4-4473-A28D-C9BCE91C6498}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:dLbls>
-          <c:dLblPos val="outEnd"/>
           <c:showLegendKey val="0"/>
-          <c:showVal val="1"/>
+          <c:showVal val="0"/>
           <c:showCatName val="0"/>
           <c:showSerName val="0"/>
           <c:showPercent val="0"/>
@@ -979,76 +746,16 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="166424991"/>
-        <c:axId val="166427871"/>
+        <c:axId val="365193039"/>
+        <c:axId val="365193519"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="166424991"/>
+        <c:axId val="365193039"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="65000"/>
-                        <a:lumOff val="35000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr lang="en-GB"/>
-                  <a:t>Number</a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="en-GB" baseline="0"/>
-                  <a:t> of Iterations</a:t>
-                </a:r>
-                <a:endParaRPr lang="en-GB"/>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-GB"/>
-            </a:p>
-          </c:txPr>
-        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -1086,7 +793,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="166427871"/>
+        <c:crossAx val="365193519"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1094,7 +801,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="166427871"/>
+        <c:axId val="365193519"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1114,61 +821,6 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="65000"/>
-                        <a:lumOff val="35000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr lang="en-GB"/>
-                  <a:t>Mean Squared Error (MSE)</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
-        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -1200,7 +852,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="166424991"/>
+        <c:crossAx val="365193039"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2340,22 +1992,22 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>7620</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>15240</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>11430</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>312420</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>556260</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>11430</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9B535FF5-82F5-368A-7638-767A7CDC0151}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{23A58024-7644-42FB-7108-22A5644A6853}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2380,23 +2032,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>579120</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>137160</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>41910</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>274320</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>441960</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>41910</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8B5A3FC5-ECC3-CBDB-CFC9-BE406EB3FBC8}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{805BE08F-35E6-8C7E-879F-2DDDE52A7D79}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2418,25 +2070,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{EDA264CB-2371-471F-A5A2-B7046C784E15}" name="Table3" displayName="Table3" ref="A1:B6" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7" tableBorderDxfId="6">
-  <autoFilter ref="A1:B6" xr:uid="{EDA264CB-2371-471F-A5A2-B7046C784E15}"/>
-  <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{ABDFE733-C989-49F7-8179-292652C3A7E5}" name="Number of Iterations" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{652ADC36-38E2-4F11-97DD-67283DBD8B6C}" name="MSE" dataDxfId="4"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{76BDDF23-E57D-4860-AE96-3D3AE711E5E3}" name="Table2" displayName="Table2" ref="A1:B6" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
-  <autoFilter ref="A1:B6" xr:uid="{76BDDF23-E57D-4860-AE96-3D3AE711E5E3}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B6">
-    <sortCondition ref="B1:B6"/>
-  </sortState>
-  <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{6B2D9E8B-ECF9-4502-9BE3-9E6793AE7D6C}" name="Number of Iterations" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{274DCDB9-B590-4F29-8207-FF1E8DFEC4A5}" name="MSE" dataDxfId="2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{2A0FDFCD-92AA-4DA1-BF45-B6DD841345FD}" name="Table4" displayName="Table4" ref="A1:C31" totalsRowShown="0" dataDxfId="0">
+  <autoFilter ref="A1:C31" xr:uid="{2A0FDFCD-92AA-4DA1-BF45-B6DD841345FD}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{8AEA0D4B-E9F5-4567-953A-1D182CFA76F1}" name="Number of Iterations" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{1F93E946-D8AD-428A-A0E9-5A7D9F258618}" name="Omega" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{37D41052-D3BF-4893-8BC5-783EDA241B2D}" name="MSE" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2738,137 +2377,429 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A51E154B-B520-40B4-8FD5-A3286721D9D2}">
-  <dimension ref="A1:C6"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D8356F9-7093-4523-A092-C1036B1CDCDE}">
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="3.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="2">
         <v>2</v>
       </c>
-      <c r="B2" s="6">
-        <v>45.213999999999999</v>
-      </c>
-      <c r="C2" s="2"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="4">
+      <c r="B2" s="4">
+        <v>42.866999999999997</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="3">
         <v>4</v>
       </c>
-      <c r="B3" s="7">
-        <v>58.094999999999999</v>
-      </c>
-      <c r="C3" s="2"/>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="3">
+      <c r="B3" s="5">
+        <v>48.762999999999998</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="2">
         <v>6</v>
       </c>
-      <c r="B4" s="7">
-        <v>64.718000000000004</v>
-      </c>
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="4">
+      <c r="B4" s="4">
+        <v>54.674999999999997</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="3">
         <v>8</v>
       </c>
-      <c r="B5" s="7">
-        <v>68.376000000000005</v>
-      </c>
-      <c r="C5" s="2"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="3">
+      <c r="B5" s="5">
+        <v>59.201000000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="2">
         <v>10</v>
       </c>
-      <c r="B6" s="7">
-        <v>70.561000000000007</v>
-      </c>
-      <c r="C6" s="2"/>
+      <c r="B6" s="4">
+        <v>62.613</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
-  <tableParts count="1">
-    <tablePart r:id="rId2"/>
-  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDB7C7F8-C35B-4306-B386-7BD9C920195C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD715877-BFE9-42BD-9D4F-1C3D61467296}">
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="1">
+      <c r="A2" s="3">
         <v>2</v>
       </c>
-      <c r="B2" s="1">
-        <v>42.866999999999997</v>
+      <c r="B2" s="7">
+        <v>45.213999999999999</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>4</v>
       </c>
-      <c r="B3" s="1">
-        <v>48.762999999999998</v>
+      <c r="B3" s="6">
+        <v>58.094999999999999</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="1">
+      <c r="A4" s="3">
         <v>6</v>
       </c>
-      <c r="B4" s="1">
-        <v>54.674999999999997</v>
+      <c r="B4" s="7">
+        <v>64.718000000000004</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>8</v>
       </c>
-      <c r="B5" s="1">
-        <v>59.201000000000001</v>
+      <c r="B5" s="6">
+        <v>68.376000000000005</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" s="1">
+      <c r="A6" s="3">
         <v>10</v>
       </c>
-      <c r="B6" s="1">
-        <v>62.613</v>
+      <c r="B6" s="7">
+        <v>70.561000000000007</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EC9FC7C-2A8B-42A3-B61F-B0C00C82015C}">
+  <dimension ref="A1:C31"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="20.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1">
+        <v>0.25</v>
+      </c>
+      <c r="C2" s="4"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
+        <v>4</v>
+      </c>
+      <c r="B3" s="1">
+        <v>0.25</v>
+      </c>
+      <c r="C3" s="5"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <v>6</v>
+      </c>
+      <c r="B4" s="1">
+        <v>0.25</v>
+      </c>
+      <c r="C4" s="4"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>8</v>
+      </c>
+      <c r="B5" s="1">
+        <v>0.25</v>
+      </c>
+      <c r="C5" s="5"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>10</v>
+      </c>
+      <c r="B6" s="1">
+        <v>0.25</v>
+      </c>
+      <c r="C6" s="4"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>2</v>
+      </c>
+      <c r="B7" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="C7" s="1"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>4</v>
+      </c>
+      <c r="B8" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="C8" s="1"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>6</v>
+      </c>
+      <c r="B9" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="C9" s="1"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="1">
+        <v>8</v>
+      </c>
+      <c r="B10" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="C10" s="1"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="1">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="C11" s="1"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="1">
+        <v>2</v>
+      </c>
+      <c r="B12" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="C12" s="1"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="1">
+        <v>4</v>
+      </c>
+      <c r="B13" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="C13" s="1"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="1">
+        <v>6</v>
+      </c>
+      <c r="B14" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="C14" s="1"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="1">
+        <v>8</v>
+      </c>
+      <c r="B15" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="C15" s="1"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="1">
+        <v>10</v>
+      </c>
+      <c r="B16" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="C16" s="1"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="1">
+        <v>2</v>
+      </c>
+      <c r="B17" s="1">
+        <v>1.25</v>
+      </c>
+      <c r="C17" s="1"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="1">
+        <v>4</v>
+      </c>
+      <c r="B18" s="1">
+        <v>1.25</v>
+      </c>
+      <c r="C18" s="1"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="1">
+        <v>6</v>
+      </c>
+      <c r="B19" s="1">
+        <v>1.25</v>
+      </c>
+      <c r="C19" s="1"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="1">
+        <v>8</v>
+      </c>
+      <c r="B20" s="1">
+        <v>1.25</v>
+      </c>
+      <c r="C20" s="1"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="1">
+        <v>10</v>
+      </c>
+      <c r="B21" s="1">
+        <v>1.25</v>
+      </c>
+      <c r="C21" s="1"/>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="1">
+        <v>2</v>
+      </c>
+      <c r="B22" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="C22" s="1"/>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="1">
+        <v>4</v>
+      </c>
+      <c r="B23" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="C23" s="1"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" s="1">
+        <v>6</v>
+      </c>
+      <c r="B24" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="C24" s="1"/>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="1">
+        <v>8</v>
+      </c>
+      <c r="B25" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="C25" s="1"/>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" s="1">
+        <v>10</v>
+      </c>
+      <c r="B26" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="C26" s="1"/>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" s="1">
+        <v>2</v>
+      </c>
+      <c r="B27" s="1">
+        <v>1.75</v>
+      </c>
+      <c r="C27" s="1"/>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" s="1">
+        <v>4</v>
+      </c>
+      <c r="B28" s="1">
+        <v>1.75</v>
+      </c>
+      <c r="C28" s="1"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" s="1">
+        <v>6</v>
+      </c>
+      <c r="B29" s="1">
+        <v>1.75</v>
+      </c>
+      <c r="C29" s="1"/>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" s="1">
+        <v>8</v>
+      </c>
+      <c r="B30" s="1">
+        <v>1.75</v>
+      </c>
+      <c r="C30" s="1"/>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" s="1">
+        <v>10</v>
+      </c>
+      <c r="B31" s="1">
+        <v>1.75</v>
+      </c>
+      <c r="C31" s="1"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>